<commit_message>
correção de entrada de dados no formulário de perdas
</commit_message>
<xml_diff>
--- a/relatorio_comissao.xlsx
+++ b/relatorio_comissao.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L16"/>
+  <dimension ref="A1:L17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1045,41 +1045,81 @@
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>204.12</v>
+      </c>
+      <c r="C16" t="n">
+        <v>29.16</v>
+      </c>
+      <c r="D16" t="n">
+        <v>29.16</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" t="n">
+        <v>29.16</v>
+      </c>
+      <c r="H16" t="n">
+        <v>29.16</v>
+      </c>
+      <c r="I16" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" t="n">
+        <v>29.16</v>
+      </c>
+      <c r="K16" t="n">
+        <v>29.16</v>
+      </c>
+      <c r="L16" t="n">
+        <v>29.16</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B16" s="1" t="n">
-        <v>3248.24</v>
-      </c>
-      <c r="C16" s="1" t="n">
-        <v>438.81</v>
-      </c>
-      <c r="D16" s="1" t="n">
-        <v>438.81</v>
-      </c>
-      <c r="E16" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F16" s="1" t="n">
+      <c r="B17" s="1" t="n">
+        <v>3452.36</v>
+      </c>
+      <c r="C17" s="1" t="n">
+        <v>467.97</v>
+      </c>
+      <c r="D17" s="1" t="n">
+        <v>467.97</v>
+      </c>
+      <c r="E17" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="1" t="n">
         <v>320.27</v>
       </c>
-      <c r="G16" s="1" t="n">
-        <v>438.81</v>
-      </c>
-      <c r="H16" s="1" t="n">
-        <v>295.1</v>
-      </c>
-      <c r="I16" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J16" s="1" t="n">
-        <v>438.81</v>
-      </c>
-      <c r="K16" s="1" t="n">
-        <v>438.81</v>
-      </c>
-      <c r="L16" s="1" t="n">
-        <v>438.81</v>
+      <c r="G17" s="1" t="n">
+        <v>467.97</v>
+      </c>
+      <c r="H17" s="1" t="n">
+        <v>324.26</v>
+      </c>
+      <c r="I17" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" s="1" t="n">
+        <v>467.97</v>
+      </c>
+      <c r="K17" s="1" t="n">
+        <v>467.97</v>
+      </c>
+      <c r="L17" s="1" t="n">
+        <v>467.97</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Migra aba Produtos para consumir dados do Supabase
</commit_message>
<xml_diff>
--- a/relatorio_comissao.xlsx
+++ b/relatorio_comissao.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L24"/>
+  <dimension ref="A1:L25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1365,41 +1365,81 @@
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
         <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>88.08</v>
+      </c>
+      <c r="C24" t="n">
+        <v>11.01</v>
+      </c>
+      <c r="D24" t="n">
+        <v>11.01</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" t="n">
+        <v>11.01</v>
+      </c>
+      <c r="G24" t="n">
+        <v>11.01</v>
+      </c>
+      <c r="H24" t="n">
+        <v>11.01</v>
+      </c>
+      <c r="I24" t="n">
+        <v>0</v>
+      </c>
+      <c r="J24" t="n">
+        <v>11.01</v>
+      </c>
+      <c r="K24" t="n">
+        <v>11.01</v>
+      </c>
+      <c r="L24" t="n">
+        <v>11.01</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="1" t="inlineStr">
+        <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B24" s="1" t="n">
-        <v>4764.24</v>
-      </c>
-      <c r="C24" s="1" t="n">
-        <v>636.78</v>
-      </c>
-      <c r="D24" s="1" t="n">
-        <v>636.78</v>
-      </c>
-      <c r="E24" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F24" s="1" t="n">
-        <v>450.51</v>
-      </c>
-      <c r="G24" s="1" t="n">
-        <v>636.78</v>
-      </c>
-      <c r="H24" s="1" t="n">
-        <v>493.06</v>
-      </c>
-      <c r="I24" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J24" s="1" t="n">
-        <v>636.78</v>
-      </c>
-      <c r="K24" s="1" t="n">
-        <v>636.78</v>
-      </c>
-      <c r="L24" s="1" t="n">
-        <v>636.78</v>
+      <c r="B25" s="1" t="n">
+        <v>4852.32</v>
+      </c>
+      <c r="C25" s="1" t="n">
+        <v>647.79</v>
+      </c>
+      <c r="D25" s="1" t="n">
+        <v>647.79</v>
+      </c>
+      <c r="E25" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" s="1" t="n">
+        <v>461.52</v>
+      </c>
+      <c r="G25" s="1" t="n">
+        <v>647.79</v>
+      </c>
+      <c r="H25" s="1" t="n">
+        <v>504.07</v>
+      </c>
+      <c r="I25" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J25" s="1" t="n">
+        <v>647.79</v>
+      </c>
+      <c r="K25" s="1" t="n">
+        <v>647.79</v>
+      </c>
+      <c r="L25" s="1" t="n">
+        <v>647.79</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update de planilha relatorio_comissao
</commit_message>
<xml_diff>
--- a/relatorio_comissao.xlsx
+++ b/relatorio_comissao.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L25"/>
+  <dimension ref="A1:L27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1365,81 +1365,161 @@
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>88.08</v>
+        <v>148.24</v>
       </c>
       <c r="C24" t="n">
-        <v>11.01</v>
+        <v>18.53</v>
       </c>
       <c r="D24" t="n">
-        <v>11.01</v>
+        <v>18.53</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
       </c>
       <c r="F24" t="n">
-        <v>11.01</v>
+        <v>18.53</v>
       </c>
       <c r="G24" t="n">
-        <v>11.01</v>
+        <v>18.53</v>
       </c>
       <c r="H24" t="n">
-        <v>11.01</v>
+        <v>18.53</v>
       </c>
       <c r="I24" t="n">
         <v>0</v>
       </c>
       <c r="J24" t="n">
-        <v>11.01</v>
+        <v>18.53</v>
       </c>
       <c r="K24" t="n">
-        <v>11.01</v>
+        <v>18.53</v>
       </c>
       <c r="L24" t="n">
-        <v>11.01</v>
+        <v>18.53</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
         <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>88.08</v>
+      </c>
+      <c r="C25" t="n">
+        <v>11.01</v>
+      </c>
+      <c r="D25" t="n">
+        <v>11.01</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" t="n">
+        <v>11.01</v>
+      </c>
+      <c r="G25" t="n">
+        <v>11.01</v>
+      </c>
+      <c r="H25" t="n">
+        <v>11.01</v>
+      </c>
+      <c r="I25" t="n">
+        <v>0</v>
+      </c>
+      <c r="J25" t="n">
+        <v>11.01</v>
+      </c>
+      <c r="K25" t="n">
+        <v>11.01</v>
+      </c>
+      <c r="L25" t="n">
+        <v>11.01</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="1" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>189.08</v>
+      </c>
+      <c r="C26" t="n">
+        <v>23.64</v>
+      </c>
+      <c r="D26" t="n">
+        <v>23.64</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" t="n">
+        <v>23.64</v>
+      </c>
+      <c r="G26" t="n">
+        <v>23.64</v>
+      </c>
+      <c r="H26" t="n">
+        <v>23.64</v>
+      </c>
+      <c r="I26" t="n">
+        <v>0</v>
+      </c>
+      <c r="J26" t="n">
+        <v>23.64</v>
+      </c>
+      <c r="K26" t="n">
+        <v>23.64</v>
+      </c>
+      <c r="L26" t="n">
+        <v>23.64</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="inlineStr">
+        <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B25" s="1" t="n">
-        <v>4852.32</v>
-      </c>
-      <c r="C25" s="1" t="n">
-        <v>647.79</v>
-      </c>
-      <c r="D25" s="1" t="n">
-        <v>647.79</v>
-      </c>
-      <c r="E25" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F25" s="1" t="n">
-        <v>461.52</v>
-      </c>
-      <c r="G25" s="1" t="n">
-        <v>647.79</v>
-      </c>
-      <c r="H25" s="1" t="n">
-        <v>504.07</v>
-      </c>
-      <c r="I25" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J25" s="1" t="n">
-        <v>647.79</v>
-      </c>
-      <c r="K25" s="1" t="n">
-        <v>647.79</v>
-      </c>
-      <c r="L25" s="1" t="n">
-        <v>647.79</v>
+      <c r="B27" s="1" t="n">
+        <v>5189.64</v>
+      </c>
+      <c r="C27" s="1" t="n">
+        <v>689.95</v>
+      </c>
+      <c r="D27" s="1" t="n">
+        <v>689.95</v>
+      </c>
+      <c r="E27" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" s="1" t="n">
+        <v>503.69</v>
+      </c>
+      <c r="G27" s="1" t="n">
+        <v>689.95</v>
+      </c>
+      <c r="H27" s="1" t="n">
+        <v>546.24</v>
+      </c>
+      <c r="I27" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J27" s="1" t="n">
+        <v>689.95</v>
+      </c>
+      <c r="K27" s="1" t="n">
+        <v>689.95</v>
+      </c>
+      <c r="L27" s="1" t="n">
+        <v>689.95</v>
       </c>
     </row>
   </sheetData>

</xml_diff>